<commit_message>
test discriminateur code DispositifMedical 9ebaddc24ef991a4517d36baf32c4fff7ff2a84f
</commit_message>
<xml_diff>
--- a/fix/slicing-type-this/ig/StructureDefinition-fr-cda-dispositif-medical.xlsx
+++ b/fix/slicing-type-this/ig/StructureDefinition-fr-cda-dispositif-medical.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-06T14:14:01+00:00</t>
+    <t>2026-10-06T20:02:10+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1425,7 +1425,7 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">profile:observation}
+    <t xml:space="preserve">value:observation.code.code}
 </t>
   </si>
   <si>
@@ -2302,7 +2302,7 @@
     <col min="25" max="25" width="18.49609375" customWidth="true" bestFit="true"/>
     <col min="26" max="26" width="67.11328125" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
-    <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
+    <col min="28" max="28" width="24.59375" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="17.65625" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>

</xml_diff>

<commit_message>
revert test discriminateur DispositifMedical a4e3102520800f76eaa38686607c01e49edf8afc
</commit_message>
<xml_diff>
--- a/fix/slicing-type-this/ig/StructureDefinition-fr-cda-dispositif-medical.xlsx
+++ b/fix/slicing-type-this/ig/StructureDefinition-fr-cda-dispositif-medical.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-06T20:02:10+00:00</t>
+    <t>2026-10-07T08:37:44+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1425,7 +1425,7 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">value:observation.code.code}
+    <t xml:space="preserve">profile:observation}
 </t>
   </si>
   <si>
@@ -2302,7 +2302,7 @@
     <col min="25" max="25" width="18.49609375" customWidth="true" bestFit="true"/>
     <col min="26" max="26" width="67.11328125" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
-    <col min="28" max="28" width="24.59375" customWidth="true" bestFit="true"/>
+    <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="17.65625" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>

</xml_diff>